<commit_message>
Improve COMET workflow sequence audits
</commit_message>
<xml_diff>
--- a/Ref-selection/___IncludedNS5ARefs.xlsx
+++ b/Ref-selection/___IncludedNS5ARefs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rshafer/Dropbox/Vistas/HCVData-blasthit-db/CSV/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kaimingtao/HIVDB/HCV-GenBank-Skills/Ref-selection/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFFD124-4BCC-7A4C-A9A8-DA2434352B8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A16ED1-A318-7E42-B415-0F7AFA2D9D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15540" yWindow="1620" windowWidth="40300" windowHeight="20720" xr2:uid="{B505863C-43B5-554D-933F-1F46B70F71B9}"/>
+    <workbookView xWindow="720" yWindow="780" windowWidth="28240" windowHeight="20820" xr2:uid="{B505863C-43B5-554D-933F-1F46B70F71B9}"/>
   </bookViews>
   <sheets>
     <sheet name="NS5A_PtGT0_Check" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="919">
   <si>
     <t>RefID</t>
   </si>
@@ -3257,8 +3257,8 @@
       <c r="H2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>23</v>
+      <c r="I2" s="1">
+        <v>1778</v>
       </c>
       <c r="J2" s="1">
         <v>448</v>

</xml_diff>